<commit_message>
Stime finali della libreria nuova con la Fr reale
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MvMS9hCRebf92ngdXubAAu
</commit_message>
<xml_diff>
--- a/dati/Libreria_nuova_Cosmap.xlsx
+++ b/dati/Libreria_nuova_Cosmap.xlsx
@@ -470,7 +470,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Stima finale: Fr indica l'esposizione al pericolo che resta dopo le misure (accesso alla zona protetta), non la frequenza del ciclo.</t>
+          <t>Stima finale: Fr resta la frequenza reale di esposizione; la gravità scende solo dove la protezione limita il danno (motivo nelle note). Con questa matrice le schede di gravità 4 restano Richieste: verificare il PL delle misure.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
         <v>3</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>1</v>
@@ -768,11 +768,11 @@
         <v>1</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -1097,14 +1097,14 @@
         <v>1</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,11 @@
 - [PROG] Visibilità della zona di lavoro dal posto di comando attraverso finestre di ispezione.</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Durante la lavorazione restare al posto operatore previsto, fuori dalla cabina.</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="n">
         <v>2</v>
       </c>
@@ -1317,14 +1321,14 @@
         <v>1</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1528,10 +1532,10 @@
         </is>
       </c>
       <c r="S9" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U9" s="2" t="n">
         <v>1</v>
@@ -1540,11 +1544,11 @@
         <v>1</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1554,7 +1558,7 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Gravità finale ridotta: il riparo trattiene i frammenti, resta il rischio di lesioni lievi.</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1645,7 @@
         <v>4</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="2" t="n">
         <v>1</v>
@@ -1650,11 +1654,11 @@
         <v>1</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -1664,7 +1668,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1756,7 @@
         <v>3</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U11" s="2" t="n">
         <v>1</v>
@@ -1761,11 +1765,11 @@
         <v>1</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
@@ -2077,20 +2081,20 @@
         <v>3</v>
       </c>
       <c r="T14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="U14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U14" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="V14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -2100,7 +2104,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare. Misura da eseguire su ogni macchina o su un modello rappresentativo.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto. Misura da eseguire su ogni macchina o su un modello rappresentativo.</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2408,7 @@
         <v>3</v>
       </c>
       <c r="T17" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U17" s="2" t="n">
         <v>1</v>
@@ -2413,11 +2417,11 @@
         <v>1</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -2505,25 +2509,29 @@
 - [PROT] Scale e piattaforme con parapetti dove l'accesso è sopraelevato.</t>
         </is>
       </c>
-      <c r="R18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Usare solo i mezzi di accesso previsti; non salire su ripari o carpenterie.</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr">
@@ -2621,7 +2629,7 @@
         <v>3</v>
       </c>
       <c r="T19" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U19" s="2" t="n">
         <v>1</v>
@@ -2630,11 +2638,11 @@
         <v>1</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
@@ -2846,7 +2854,7 @@
         <v>4</v>
       </c>
       <c r="T21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U21" s="2" t="n">
         <v>1</v>
@@ -2855,11 +2863,11 @@
         <v>1</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -2869,7 +2877,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare. Requisito nuovo del Regolamento 2023/1230 (protezione contro la corruzione).</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto. Requisito nuovo del Regolamento 2023/1230 (protezione contro la corruzione).</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2967,7 @@
         <v>4</v>
       </c>
       <c r="T22" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U22" s="2" t="n">
         <v>1</v>
@@ -2968,11 +2976,11 @@
         <v>1</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -2982,7 +2990,7 @@
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare. Regolamento 2023/1230: il sistema di comando deve resistere anche ad azioni malevole e tracciare gli interventi sul software di sicurezza.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto. Regolamento 2023/1230: il sistema di comando deve resistere anche ad azioni malevole e tracciare gli interventi sul software di sicurezza.</t>
         </is>
       </c>
     </row>
@@ -3061,12 +3069,16 @@
 - [PROG] Colori dei pulsanti e degli indicatori secondo le regole dell'equipaggiamento elettrico.</t>
         </is>
       </c>
-      <c r="R23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Prima di azionare un comando verificarne la funzione sul pannello; i selettori dei modi sono riservati a personale autorizzato.</t>
+        </is>
+      </c>
       <c r="S23" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T23" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U23" s="2" t="n">
         <v>1</v>
@@ -3075,11 +3087,11 @@
         <v>1</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -3175,7 +3187,7 @@
         <v>4</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U24" s="2" t="n">
         <v>1</v>
@@ -3184,11 +3196,11 @@
         <v>1</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
@@ -3198,7 +3210,7 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3274,12 +3286,16 @@
           <t>- [PROG] Comando di arresto che ferma tutte le funzioni pericolose con priorità sull'avviamento (categoria 0 o 1).</t>
         </is>
       </c>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Per fermare la macchina in condizioni normali usare il comando di arresto, non l'arresto di emergenza.</t>
+        </is>
+      </c>
       <c r="S25" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T25" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U25" s="2" t="n">
         <v>1</v>
@@ -3288,11 +3304,11 @@
         <v>1</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y25" s="2" t="inlineStr">
@@ -3387,7 +3403,7 @@
         <v>4</v>
       </c>
       <c r="T26" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U26" s="2" t="n">
         <v>1</v>
@@ -3396,11 +3412,11 @@
         <v>1</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -3410,7 +3426,7 @@
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3512,7 @@
         <v>4</v>
       </c>
       <c r="T27" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U27" s="2" t="n">
         <v>1</v>
@@ -3505,11 +3521,11 @@
         <v>1</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y27" s="2" t="inlineStr">
@@ -3519,7 +3535,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3622,7 @@
         <v>4</v>
       </c>
       <c r="T28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U28" s="2" t="n">
         <v>1</v>
@@ -3615,11 +3631,11 @@
         <v>1</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y28" s="2" t="inlineStr">
@@ -3629,7 +3645,7 @@
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3734,7 @@
         <v>4</v>
       </c>
       <c r="T29" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U29" s="2" t="n">
         <v>1</v>
@@ -3727,11 +3743,11 @@
         <v>1</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y29" s="2" t="inlineStr">
@@ -3741,7 +3757,7 @@
       </c>
       <c r="Z29" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3846,7 @@
         <v>4</v>
       </c>
       <c r="T30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U30" s="2" t="n">
         <v>1</v>
@@ -3839,11 +3855,11 @@
         <v>1</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y30" s="2" t="inlineStr">
@@ -3853,7 +3869,7 @@
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3957,7 @@
         <v>4</v>
       </c>
       <c r="T31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U31" s="2" t="n">
         <v>1</v>
@@ -3950,11 +3966,11 @@
         <v>1</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y31" s="2" t="inlineStr">
@@ -3964,7 +3980,7 @@
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4057,11 @@
           <t>- [PROG] Messa a terra delle parti metalliche e delle condotte di aspirazione per scaricare le cariche elettrostatiche.</t>
         </is>
       </c>
-      <c r="R32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Non scollegare i collegamenti di terra delle condotte e delle parti metalliche.</t>
+        </is>
+      </c>
       <c r="S32" s="2" t="n">
         <v>2</v>
       </c>
@@ -4052,14 +4072,14 @@
         <v>1</v>
       </c>
       <c r="V32" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W32" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y32" s="2" t="inlineStr">
@@ -4145,7 +4165,11 @@
           <t>- [PROG] Nessuna sorgente significativa di radiazioni; motori e inverter conformi alle norme EMC.</t>
         </is>
       </c>
-      <c r="R33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Le persone portatrici di dispositivi medici impiantati devono consultare il medico prima di lavorare vicino a motori e quadri.</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="n">
         <v>2</v>
       </c>
@@ -4156,14 +4180,14 @@
         <v>1</v>
       </c>
       <c r="V33" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W33" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X33" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y33" s="2" t="inlineStr">
@@ -4249,12 +4273,16 @@
           <t>- [PROG] Immunità ai disturbi per ambiente industriale; cablaggi schermati e separati dalla potenza.</t>
         </is>
       </c>
-      <c r="R34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Non installare vicino alla macchina apparecchi che emettono forti disturbi elettromagnetici (saldatrici, trasmettitori).</t>
+        </is>
+      </c>
       <c r="S34" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T34" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U34" s="2" t="n">
         <v>1</v>
@@ -4263,11 +4291,11 @@
         <v>1</v>
       </c>
       <c r="W34" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y34" s="2" t="inlineStr">
@@ -4473,7 +4501,7 @@
         <v>4</v>
       </c>
       <c r="T36" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U36" s="2" t="n">
         <v>1</v>
@@ -4482,11 +4510,11 @@
         <v>1</v>
       </c>
       <c r="W36" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y36" s="2" t="inlineStr">
@@ -4496,7 +4524,7 @@
       </c>
       <c r="Z36" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -4572,12 +4600,16 @@
           <t>- [INFO] Testi e messaggi sul pannello nella lingua del paese di utilizzo; preferiti simboli e pittogrammi.</t>
         </is>
       </c>
-      <c r="R37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>Leggere i messaggi del pannello prima di intervenire; se non sono chiari consultare il manuale.</t>
+        </is>
+      </c>
       <c r="S37" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T37" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U37" s="2" t="n">
         <v>1</v>
@@ -4586,11 +4618,11 @@
         <v>1</v>
       </c>
       <c r="W37" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X37" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y37" s="2" t="inlineStr">
@@ -4677,12 +4709,16 @@
           <t>- [PROG] Il pannello mostra stato della macchina, modo attivo, allarmi e causa degli arresti in modo chiaro.</t>
         </is>
       </c>
-      <c r="R38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>In caso di allarme leggere la causa sul pannello e seguire la procedura del manuale prima di riavviare.</t>
+        </is>
+      </c>
       <c r="S38" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T38" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U38" s="2" t="n">
         <v>1</v>
@@ -4691,11 +4727,11 @@
         <v>1</v>
       </c>
       <c r="W38" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X38" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y38" s="2" t="inlineStr">
@@ -4792,7 +4828,7 @@
         <v>4</v>
       </c>
       <c r="T39" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U39" s="2" t="n">
         <v>1</v>
@@ -4801,11 +4837,11 @@
         <v>1</v>
       </c>
       <c r="W39" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X39" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y39" s="2" t="inlineStr">
@@ -4815,7 +4851,7 @@
       </c>
       <c r="Z39" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4937,7 @@
         <v>4</v>
       </c>
       <c r="T40" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U40" s="2" t="n">
         <v>1</v>
@@ -4910,11 +4946,11 @@
         <v>1</v>
       </c>
       <c r="W40" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X40" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y40" s="2" t="inlineStr">
@@ -4924,7 +4960,7 @@
       </c>
       <c r="Z40" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5106,12 +5142,16 @@
 - [INFO] Manuale in formato digitale, con copia cartacea su richiesta del cliente al momento dell'acquisto.</t>
         </is>
       </c>
-      <c r="R42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Conservare il manuale vicino alla macchina e renderlo disponibile a chi la usa e la manutiene.</t>
+        </is>
+      </c>
       <c r="S42" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T42" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U42" s="2" t="n">
         <v>1</v>
@@ -5120,11 +5160,11 @@
         <v>1</v>
       </c>
       <c r="W42" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
@@ -5211,12 +5251,16 @@
 - [INFO] Copia della dichiarazione UE di conformità o indirizzo dove consultarla.</t>
         </is>
       </c>
-      <c r="R43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Leggere il manuale prima di usare, regolare o manutenere la macchina.</t>
+        </is>
+      </c>
       <c r="S43" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T43" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U43" s="2" t="n">
         <v>1</v>
@@ -5225,11 +5269,11 @@
         <v>1</v>
       </c>
       <c r="W43" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y43" s="2" t="inlineStr">
@@ -5432,7 +5476,7 @@
         <v>4</v>
       </c>
       <c r="T45" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U45" s="2" t="n">
         <v>1</v>
@@ -5441,11 +5485,11 @@
         <v>1</v>
       </c>
       <c r="W45" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y45" s="2" t="inlineStr">
@@ -5455,7 +5499,7 @@
       </c>
       <c r="Z45" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5586,7 @@
         <v>4</v>
       </c>
       <c r="T46" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U46" s="2" t="n">
         <v>1</v>
@@ -5551,11 +5595,11 @@
         <v>1</v>
       </c>
       <c r="W46" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
@@ -5565,7 +5609,7 @@
       </c>
       <c r="Z46" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5700,7 @@
         <v>4</v>
       </c>
       <c r="T47" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U47" s="2" t="n">
         <v>1</v>
@@ -5665,11 +5709,11 @@
         <v>1</v>
       </c>
       <c r="W47" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X47" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y47" s="2" t="inlineStr">
@@ -5679,7 +5723,7 @@
       </c>
       <c r="Z47" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5766,7 +5810,7 @@
         <v>4</v>
       </c>
       <c r="T48" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U48" s="2" t="n">
         <v>1</v>
@@ -5775,11 +5819,11 @@
         <v>1</v>
       </c>
       <c r="W48" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr">
@@ -5789,7 +5833,7 @@
       </c>
       <c r="Z48" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5921,7 @@
         <v>4</v>
       </c>
       <c r="T49" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U49" s="2" t="n">
         <v>1</v>
@@ -5886,11 +5930,11 @@
         <v>1</v>
       </c>
       <c r="W49" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X49" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y49" s="2" t="inlineStr">
@@ -5900,7 +5944,7 @@
       </c>
       <c r="Z49" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -5977,12 +6021,16 @@
           <t>- [PROG] Porte di dimensioni adeguate al passaggio di una persona con attrezzi; nessun ostacolo all'ingresso.</t>
         </is>
       </c>
-      <c r="R50" s="2" t="inlineStr"/>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Prima di entrare nella cella per manutenzione o pulizia arrestare e sezionare la macchina.</t>
+        </is>
+      </c>
       <c r="S50" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T50" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U50" s="2" t="n">
         <v>1</v>
@@ -5991,11 +6039,11 @@
         <v>1</v>
       </c>
       <c r="W50" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X50" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y50" s="2" t="inlineStr">
@@ -6093,7 +6141,7 @@
         <v>4</v>
       </c>
       <c r="T51" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U51" s="2" t="n">
         <v>1</v>
@@ -6102,11 +6150,11 @@
         <v>1</v>
       </c>
       <c r="W51" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X51" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y51" s="2" t="inlineStr">
@@ -6116,7 +6164,7 @@
       </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -6205,7 +6253,7 @@
         <v>4</v>
       </c>
       <c r="T52" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U52" s="2" t="n">
         <v>1</v>
@@ -6214,11 +6262,11 @@
         <v>1</v>
       </c>
       <c r="W52" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y52" s="2" t="inlineStr">
@@ -6228,7 +6276,7 @@
       </c>
       <c r="Z52" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6363,7 @@
         <v>4</v>
       </c>
       <c r="T53" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U53" s="2" t="n">
         <v>1</v>
@@ -6324,11 +6372,11 @@
         <v>1</v>
       </c>
       <c r="W53" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X53" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y53" s="2" t="inlineStr">
@@ -6338,7 +6386,7 @@
       </c>
       <c r="Z53" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6472,7 @@
         <v>4</v>
       </c>
       <c r="T54" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U54" s="2" t="n">
         <v>1</v>
@@ -6433,11 +6481,11 @@
         <v>1</v>
       </c>
       <c r="W54" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
@@ -6447,7 +6495,7 @@
       </c>
       <c r="Z54" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6582,7 @@
         <v>4</v>
       </c>
       <c r="T55" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U55" s="2" t="n">
         <v>1</v>
@@ -6543,11 +6591,11 @@
         <v>1</v>
       </c>
       <c r="W55" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X55" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y55" s="2" t="inlineStr">
@@ -6557,7 +6605,7 @@
       </c>
       <c r="Z55" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -6646,7 +6694,7 @@
         <v>3</v>
       </c>
       <c r="T56" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U56" s="2" t="n">
         <v>1</v>
@@ -6655,11 +6703,11 @@
         <v>1</v>
       </c>
       <c r="W56" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y56" s="2" t="inlineStr">
@@ -6746,12 +6794,16 @@
 - [PROT] Cabina chiusa che trattiene pezzi e frammenti proiettati.</t>
         </is>
       </c>
-      <c r="R57" s="2" t="inlineStr"/>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Non aprire la cabina durante la smerigliatura; usare occhiali di protezione quando si interviene dopo la lavorazione.</t>
+        </is>
+      </c>
       <c r="S57" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T57" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U57" s="2" t="n">
         <v>1</v>
@@ -6760,11 +6812,11 @@
         <v>1</v>
       </c>
       <c r="W57" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X57" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y57" s="2" t="inlineStr">
@@ -6863,7 +6915,7 @@
         <v>3</v>
       </c>
       <c r="T58" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U58" s="2" t="n">
         <v>1</v>
@@ -6872,11 +6924,11 @@
         <v>1</v>
       </c>
       <c r="W58" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X58" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y58" s="2" t="inlineStr">
@@ -6970,10 +7022,10 @@
         </is>
       </c>
       <c r="S59" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T59" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U59" s="2" t="n">
         <v>1</v>
@@ -6982,7 +7034,7 @@
         <v>1</v>
       </c>
       <c r="W59" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X59" s="2" t="inlineStr">
         <is>
@@ -6996,7 +7048,7 @@
       </c>
       <c r="Z59" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Gravità finale ridotta: cabina non combustibile e parascintille limitano l'estensione dell'incendio.</t>
         </is>
       </c>
     </row>
@@ -7082,7 +7134,7 @@
         <v>3</v>
       </c>
       <c r="T60" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U60" s="2" t="n">
         <v>1</v>
@@ -7091,11 +7143,11 @@
         <v>1</v>
       </c>
       <c r="W60" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X60" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y60" s="2" t="inlineStr">
@@ -7193,7 +7245,7 @@
         <v>3</v>
       </c>
       <c r="T61" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U61" s="2" t="n">
         <v>1</v>
@@ -7202,11 +7254,11 @@
         <v>1</v>
       </c>
       <c r="W61" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y61" s="2" t="inlineStr">
@@ -7293,12 +7345,16 @@
 - [PROT] Cabina chiusa che trattiene pezzi e frammenti proiettati.</t>
         </is>
       </c>
-      <c r="R62" s="2" t="inlineStr"/>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>Non aprire la cabina durante la lucidatura; usare occhiali di protezione quando si interviene dopo la lavorazione.</t>
+        </is>
+      </c>
       <c r="S62" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T62" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U62" s="2" t="n">
         <v>1</v>
@@ -7307,11 +7363,11 @@
         <v>1</v>
       </c>
       <c r="W62" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y62" s="2" t="inlineStr">
@@ -7398,12 +7454,16 @@
           <t>- [PROT] Carter fissi sulle trasmissioni a cinghia.</t>
         </is>
       </c>
-      <c r="R63" s="2" t="inlineStr"/>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Rimontare i carter delle trasmissioni dopo ogni intervento.</t>
+        </is>
+      </c>
       <c r="S63" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T63" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U63" s="2" t="n">
         <v>1</v>
@@ -7412,11 +7472,11 @@
         <v>1</v>
       </c>
       <c r="W63" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y63" s="2" t="inlineStr">
@@ -7514,7 +7574,7 @@
         <v>3</v>
       </c>
       <c r="T64" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U64" s="2" t="n">
         <v>1</v>
@@ -7523,11 +7583,11 @@
         <v>1</v>
       </c>
       <c r="W64" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X64" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y64" s="2" t="inlineStr">
@@ -7620,10 +7680,10 @@
         </is>
       </c>
       <c r="S65" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T65" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U65" s="2" t="n">
         <v>1</v>
@@ -7632,7 +7692,7 @@
         <v>1</v>
       </c>
       <c r="W65" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X65" s="2" t="inlineStr">
         <is>
@@ -7646,7 +7706,7 @@
       </c>
       <c r="Z65" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Gravità finale ridotta: vasche metalliche e pulizia limitano l'estensione dell'incendio.</t>
         </is>
       </c>
     </row>
@@ -7733,7 +7793,7 @@
         <v>2</v>
       </c>
       <c r="T66" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U66" s="2" t="n">
         <v>1</v>
@@ -7742,7 +7802,7 @@
         <v>1</v>
       </c>
       <c r="W66" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X66" s="2" t="inlineStr">
         <is>
@@ -7834,12 +7894,16 @@
 - [PROG] Attrezzature di carico che centrano il pezzo senza forzare.</t>
         </is>
       </c>
-      <c r="R67" s="2" t="inlineStr"/>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Fare pause e alternare le mansioni quando il carico manuale è continuo.</t>
+        </is>
+      </c>
       <c r="S67" s="2" t="n">
         <v>2</v>
       </c>
       <c r="T67" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U67" s="2" t="n">
         <v>2</v>
@@ -7848,11 +7912,11 @@
         <v>1</v>
       </c>
       <c r="W67" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="X67" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y67" s="2" t="inlineStr">
@@ -7951,7 +8015,7 @@
         <v>4</v>
       </c>
       <c r="T68" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U68" s="2" t="n">
         <v>1</v>
@@ -7960,11 +8024,11 @@
         <v>1</v>
       </c>
       <c r="W68" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X68" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y68" s="2" t="inlineStr">
@@ -7974,7 +8038,7 @@
       </c>
       <c r="Z68" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -8051,12 +8115,16 @@
           <t>- [PROT] Trasmissione della tavola chiusa da carter fissi.</t>
         </is>
       </c>
-      <c r="R69" s="2" t="inlineStr"/>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>Rimontare il carter della trasmissione della tavola dopo ogni intervento.</t>
+        </is>
+      </c>
       <c r="S69" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T69" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U69" s="2" t="n">
         <v>1</v>
@@ -8065,11 +8133,11 @@
         <v>1</v>
       </c>
       <c r="W69" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X69" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y69" s="2" t="inlineStr">
@@ -8166,7 +8234,7 @@
         <v>4</v>
       </c>
       <c r="T70" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U70" s="2" t="n">
         <v>1</v>
@@ -8175,11 +8243,11 @@
         <v>1</v>
       </c>
       <c r="W70" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X70" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y70" s="2" t="inlineStr">
@@ -8189,7 +8257,7 @@
       </c>
       <c r="Z70" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -8277,7 +8345,7 @@
         <v>4</v>
       </c>
       <c r="T71" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U71" s="2" t="n">
         <v>1</v>
@@ -8286,11 +8354,11 @@
         <v>1</v>
       </c>
       <c r="W71" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X71" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y71" s="2" t="inlineStr">
@@ -8300,7 +8368,7 @@
       </c>
       <c r="Z71" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -8377,12 +8445,16 @@
           <t>- [PROG] Bloccaggio meccanico del pallet in posizione; nessun movimento per gravità.</t>
         </is>
       </c>
-      <c r="R72" s="2" t="inlineStr"/>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Dopo una mancanza di energia verificare che il pallet sia bloccato prima di intervenire.</t>
+        </is>
+      </c>
       <c r="S72" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T72" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U72" s="2" t="n">
         <v>1</v>
@@ -8391,11 +8463,11 @@
         <v>1</v>
       </c>
       <c r="W72" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X72" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y72" s="2" t="inlineStr">
@@ -8491,7 +8563,7 @@
         <v>4</v>
       </c>
       <c r="T73" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U73" s="2" t="n">
         <v>1</v>
@@ -8500,11 +8572,11 @@
         <v>1</v>
       </c>
       <c r="W73" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X73" s="2" t="inlineStr">
         <is>
-          <t>Suggerite</t>
+          <t>Richieste</t>
         </is>
       </c>
       <c r="Y73" s="2" t="inlineStr">
@@ -8514,7 +8586,7 @@
       </c>
       <c r="Z73" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Con la Fr reale la matrice dà Richieste per la gravità 4 anche con tutte le protezioni: verificare che le misure abbiano il PL richiesto.</t>
         </is>
       </c>
     </row>
@@ -8597,7 +8669,7 @@
         <v>2</v>
       </c>
       <c r="T74" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U74" s="2" t="n">
         <v>1</v>
@@ -8606,7 +8678,7 @@
         <v>1</v>
       </c>
       <c r="W74" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X74" s="2" t="inlineStr">
         <is>
@@ -8698,12 +8770,16 @@
 - [PROT] Pulsante di arresto di emergenza lungo il trasportatore.</t>
         </is>
       </c>
-      <c r="R75" s="2" t="inlineStr"/>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>Non rimuovere i ripari del trasportatore e non intervenire con il nastro in movimento.</t>
+        </is>
+      </c>
       <c r="S75" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T75" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U75" s="2" t="n">
         <v>1</v>
@@ -8712,11 +8788,11 @@
         <v>1</v>
       </c>
       <c r="W75" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X75" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y75" s="2" t="inlineStr">
@@ -8802,12 +8878,16 @@
           <t>- [PROT] Carter fissi apribili solo con attrezzo.</t>
         </is>
       </c>
-      <c r="R76" s="2" t="inlineStr"/>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>Rimontare i carter del trasportatore dopo ogni intervento.</t>
+        </is>
+      </c>
       <c r="S76" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T76" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U76" s="2" t="n">
         <v>1</v>
@@ -8816,11 +8896,11 @@
         <v>1</v>
       </c>
       <c r="W76" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X76" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y76" s="2" t="inlineStr">
@@ -8916,7 +8996,7 @@
         <v>2</v>
       </c>
       <c r="T77" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U77" s="2" t="n">
         <v>1</v>
@@ -8925,7 +9005,7 @@
         <v>1</v>
       </c>
       <c r="W77" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="X77" s="2" t="inlineStr">
         <is>
@@ -9025,7 +9105,7 @@
         <v>3</v>
       </c>
       <c r="T78" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U78" s="2" t="n">
         <v>1</v>
@@ -9034,11 +9114,11 @@
         <v>1</v>
       </c>
       <c r="W78" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X78" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y78" s="2" t="inlineStr">
@@ -9130,7 +9210,7 @@
         <v>2</v>
       </c>
       <c r="T79" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U79" s="2" t="n">
         <v>1</v>
@@ -9139,7 +9219,7 @@
         <v>1</v>
       </c>
       <c r="W79" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X79" s="2" t="inlineStr">
         <is>
@@ -9236,7 +9316,7 @@
         <v>2</v>
       </c>
       <c r="T80" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U80" s="2" t="n">
         <v>1</v>
@@ -9245,7 +9325,7 @@
         <v>1</v>
       </c>
       <c r="W80" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X80" s="2" t="inlineStr">
         <is>
@@ -9337,12 +9417,16 @@
 - [PROG] Valvole che mantengono in posizione gli attuatori che trattengono carichi.</t>
         </is>
       </c>
-      <c r="R81" s="2" t="inlineStr"/>
+      <c r="R81" s="2" t="inlineStr">
+        <is>
+          <t>Dopo una mancanza di aria compressa verificare la posizione degli attuatori prima di riavviare.</t>
+        </is>
+      </c>
       <c r="S81" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T81" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U81" s="2" t="n">
         <v>1</v>
@@ -9351,11 +9435,11 @@
         <v>1</v>
       </c>
       <c r="W81" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X81" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y81" s="2" t="inlineStr">
@@ -9443,12 +9527,16 @@
 - [PROT] Cilindri accessibili solo dentro la cella interbloccata.</t>
         </is>
       </c>
-      <c r="R82" s="2" t="inlineStr"/>
+      <c r="R82" s="2" t="inlineStr">
+        <is>
+          <t>Prima di intervenire sui cilindri scaricare la pressione residua.</t>
+        </is>
+      </c>
       <c r="S82" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T82" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U82" s="2" t="n">
         <v>1</v>
@@ -9457,11 +9545,11 @@
         <v>1</v>
       </c>
       <c r="W82" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X82" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y82" s="2" t="inlineStr">
@@ -9552,7 +9640,7 @@
         <v>2</v>
       </c>
       <c r="T83" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U83" s="2" t="n">
         <v>1</v>
@@ -9561,7 +9649,7 @@
         <v>1</v>
       </c>
       <c r="W83" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X83" s="2" t="inlineStr">
         <is>
@@ -9661,7 +9749,7 @@
         <v>3</v>
       </c>
       <c r="T84" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U84" s="2" t="n">
         <v>1</v>
@@ -9670,11 +9758,11 @@
         <v>1</v>
       </c>
       <c r="W84" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="X84" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y84" s="2" t="inlineStr">
@@ -9767,10 +9855,10 @@
         </is>
       </c>
       <c r="S85" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T85" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U85" s="2" t="n">
         <v>1</v>
@@ -9779,7 +9867,7 @@
         <v>1</v>
       </c>
       <c r="W85" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X85" s="2" t="inlineStr">
         <is>
@@ -9793,7 +9881,7 @@
       </c>
       <c r="Z85" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare.</t>
+          <t>Stime proposte, da validare. Gravità finale ridotta: parascintille e filtro non combustibile limitano l'estensione dell'incendio.</t>
         </is>
       </c>
     </row>
@@ -9876,10 +9964,10 @@
         </is>
       </c>
       <c r="S86" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T86" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U86" s="2" t="n">
         <v>1</v>
@@ -9888,7 +9976,7 @@
         <v>1</v>
       </c>
       <c r="W86" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X86" s="2" t="inlineStr">
         <is>
@@ -9902,7 +9990,7 @@
       </c>
       <c r="Z86" s="2" t="inlineStr">
         <is>
-          <t>Stime proposte, da validare. Applicabile solo se si lavorano metalli che producono polveri esplosive: altrimenti segnare non applicabile.</t>
+          <t>Stime proposte, da validare. Gravità finale ridotta: le protezioni contro l'esplosione limitano gli effetti verso le persone. Applicabile solo se si lavorano metalli che producono polveri esplosive: altrimenti segnare non applicabile.</t>
         </is>
       </c>
     </row>
@@ -9979,12 +10067,16 @@
 - [PROT] Consenso alla lavorazione solo con aspirazione in funzione.</t>
         </is>
       </c>
-      <c r="R87" s="2" t="inlineStr"/>
+      <c r="R87" s="2" t="inlineStr">
+        <is>
+          <t>Non lavorare con l'aspirazione spenta o guasta; controllare periodicamente l'efficienza dei filtri.</t>
+        </is>
+      </c>
       <c r="S87" s="2" t="n">
         <v>3</v>
       </c>
       <c r="T87" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U87" s="2" t="n">
         <v>1</v>
@@ -9993,11 +10085,11 @@
         <v>1</v>
       </c>
       <c r="W87" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X87" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Suggerite</t>
         </is>
       </c>
       <c r="Y87" s="2" t="inlineStr">
@@ -10093,7 +10185,7 @@
         <v>2</v>
       </c>
       <c r="T88" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U88" s="2" t="n">
         <v>1</v>
@@ -10102,7 +10194,7 @@
         <v>1</v>
       </c>
       <c r="W88" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X88" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Soggetti esposti (RESS 1.1.1 c e d): figure, figure della macchina, campo nelle schede
- Libreria: 8 figure standard (operatori e persone esposte), modificabili da amministrazione.
- Macchina: figure con la descrizione concreta per la commessa (es. mulettista nella corsia adiacente).
- Schede modello e dell'analisi: campo Soggetti esposti, copiato con la scheda; le figure usate
  si aggiungono alla macchina con la descrizione standard.
- Controllo prima della verifica: schede con pericoli senza soggetti.
- Valutazione dei rischi in Word: capitolo Soggetti e riga Soggetti esposti in ogni scheda.
- Libreria NL: soggetti precompilati (colonna facoltativa nell'Excel, letta dall'importazione).
- Comando completa_soggetti per le analisi in bozza nate prima di questa modifica.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Libreria_nuova_Cosmap.xlsx
+++ b/dati/Libreria_nuova_Cosmap.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -520,46 +520,60 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Edizioni e stato di armonizzazione delle norme vanno verificati sulla GUUE.</t>
+          <t>Soggetti esposti proposti in base a condizioni operative e pericoli (ultima colonna del foglio Libreria):</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>operatori secondo il RESS 1.1.1 d) e persone esposte secondo il RESS 1.1.1 c).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Requisiti senza scheda (di regola non applicabili, da dichiarare nell'applicabilità):</t>
+          <t>Edizioni e stato di armonizzazione delle norme vanno verificati sulla GUUE.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1.1.8 Sedile; 1.4.2.3 Ripari regolabili; 1.5.9 Vibrazioni; 1.5.10 Radiazioni; 1.5.11 Radiazioni esterne;</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1.5.12 Radiazioni laser; 1.5.16 Fulmine.</t>
+          <t>Requisiti senza scheda (di regola non applicabili, da dichiarare nell'applicabilità):</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1.1.8 Sedile; 1.4.2.3 Ripari regolabili; 1.5.9 Vibrazioni; 1.5.10 Radiazioni; 1.5.11 Radiazioni esterne;</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>1.5.12 Radiazioni laser; 1.5.16 Fulmine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Fogli: Libreria (schede), Misure, Moduli, RESS-Regolamento, Norme, Pericoli, Metodo, Punti aperti.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Il file si rigenera con: python dati/genera_libreria_nuova.py</t>
         </is>
@@ -576,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z89"/>
+  <dimension ref="A1:AA89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -605,6 +619,7 @@
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="40" customWidth="1" min="25" max="25"/>
     <col width="35" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -736,6 +751,11 @@
       <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Note di revisione</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Soggetti esposti</t>
         </is>
       </c>
     </row>
@@ -810,6 +830,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -885,6 +906,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -995,6 +1017,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1102,6 +1129,11 @@
       <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio; Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -1215,6 +1247,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>Installatore / collaudatore</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1320,6 +1357,11 @@
       <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
         </is>
       </c>
     </row>
@@ -1399,6 +1441,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1506,6 +1549,11 @@
       <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Installatore / collaudatore</t>
         </is>
       </c>
     </row>
@@ -1612,6 +1660,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1723,6 +1776,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1831,6 +1889,11 @@
       <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore elettrico; Installatore / collaudatore</t>
         </is>
       </c>
     </row>
@@ -1944,6 +2007,11 @@
           <t>Valori da misurare sul primo impianto della serie. Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2054,6 +2122,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico; Addetto alle pulizie; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2164,6 +2237,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2272,6 +2350,11 @@
       <c r="Z16" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -2351,6 +2434,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2463,6 +2547,11 @@
           <t>Nuovo requisito del Regolamento: verificare le scelte con il fornitore del PLC. Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2574,6 +2663,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2684,6 +2778,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2793,6 +2892,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2901,6 +3005,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3010,6 +3119,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3120,6 +3234,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3227,6 +3346,11 @@
       <c r="Z25" s="2" t="inlineStr">
         <is>
           <t>Valutare caso per caso quando l'impianto entra in un insieme. Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Installatore / collaudatore</t>
         </is>
       </c>
     </row>
@@ -3340,6 +3464,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di attrezzaggio; Programmatore; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3450,6 +3579,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3558,6 +3692,11 @@
       <c r="Z28" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio; Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -3633,6 +3772,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3740,6 +3880,11 @@
       <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -3854,6 +3999,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3964,6 +4114,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4070,6 +4225,11 @@
       <c r="Z33" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
         </is>
       </c>
     </row>
@@ -4183,6 +4343,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4294,6 +4459,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4404,6 +4574,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4512,6 +4687,11 @@
       <c r="Z37" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
         </is>
       </c>
     </row>
@@ -4620,6 +4800,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4727,6 +4912,11 @@
       <c r="Z39" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
         </is>
       </c>
     </row>
@@ -4840,6 +5030,11 @@
           <t>Decidere se il consenso dall'aspirazione è di serie. Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4950,6 +5145,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5057,6 +5257,11 @@
       <c r="Z42" s="2" t="inlineStr">
         <is>
           <t>Punto aperto: classificazione delle polveri da ottone e abrasivo. Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
         </is>
       </c>
     </row>
@@ -5170,6 +5375,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>Addetto alle pulizie</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5275,6 +5485,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5386,6 +5601,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5492,6 +5712,11 @@
       <c r="Z46" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
         </is>
       </c>
     </row>
@@ -5599,6 +5824,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5704,6 +5934,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5814,6 +6049,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio; Programmatore</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5921,6 +6161,11 @@
       <c r="Z50" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -6034,6 +6279,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di attrezzaggio; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6144,6 +6394,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6254,6 +6509,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6363,6 +6623,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6471,6 +6736,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6580,6 +6850,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di attrezzaggio; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6689,6 +6964,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6798,6 +7078,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6906,6 +7191,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7013,6 +7303,11 @@
       <c r="Z60" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA60" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
         </is>
       </c>
     </row>
@@ -7126,6 +7421,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7236,6 +7536,11 @@
           <t>Rischio incendio da considerare con attenzione nella zona di pulitura. Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7345,6 +7650,11 @@
           <t>Punto aperto: classificazione delle polveri di lucidatura. Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7453,6 +7763,11 @@
       <c r="Z64" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA64" s="2" t="inlineStr">
+        <is>
+          <t>Addetto alle pulizie</t>
         </is>
       </c>
     </row>
@@ -7566,6 +7881,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA65" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Operatore di attrezzaggio</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7673,6 +7993,11 @@
       <c r="Z66" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA66" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -7785,6 +8110,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA67" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7895,6 +8225,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA68" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8005,6 +8340,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA69" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di attrezzaggio; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8111,6 +8451,11 @@
       <c r="Z70" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA70" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
         </is>
       </c>
     </row>
@@ -8223,6 +8568,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA71" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore elettrico</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8333,6 +8683,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA72" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore elettrico</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8443,6 +8798,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA73" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore elettrico; Addetto alle pulizie</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8546,6 +8906,11 @@
       <c r="Z74" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA74" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore elettrico; Terzi di passaggio</t>
         </is>
       </c>
     </row>
@@ -8653,6 +9018,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA75" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8763,6 +9133,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA76" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -8868,6 +9243,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA77" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -8972,6 +9352,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA78" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9082,6 +9467,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA79" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9192,6 +9582,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA80" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9299,6 +9694,11 @@
       <c r="Z81" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA81" s="2" t="inlineStr">
+        <is>
+          <t>Manutentore meccanico; Addetto alle pulizie</t>
         </is>
       </c>
     </row>
@@ -9405,6 +9805,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico; Terzi di passaggio</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9509,6 +9914,11 @@
           <t>Stima proposta, da validare.</t>
         </is>
       </c>
+      <c r="AA83" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9612,6 +10022,11 @@
       <c r="Z84" s="2" t="inlineStr">
         <is>
           <t>Stima proposta, da validare.</t>
+        </is>
+      </c>
+      <c r="AA84" s="2" t="inlineStr">
+        <is>
+          <t>Operatore di conduzione; Manutentore meccanico; Terzi di passaggio</t>
         </is>
       </c>
     </row>
@@ -9691,6 +10106,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -9763,6 +10179,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9836,6 +10253,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9908,6 +10326,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -9980,6 +10399,7 @@
           <t>Scheda descrittiva, senza stima del rischio.</t>
         </is>
       </c>
+      <c r="AA89" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cl ed esito nella scheda modello; pericoli secondo il registro EN ISO 12100
La scheda modello mostra Cl = Fr + Pr + Av con l'esito della matrice, come nell'analisi.
L'elenco dei pericoli è rigenerato dal registro interno EN ISO 12100 (46 voci a tre livelli);
la migrazione 0014 converte i pericoli di libreria e schede con tabelle di corrispondenza
ed elimina le voci precedenti. Generatore ed Excel NL usano i nuovi codici.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MvMS9hCRebf92ngdXubAAu
</commit_message>
<xml_diff>
--- a/dati/Libreria_nuova_Cosmap.xlsx
+++ b/dati/Libreria_nuova_Cosmap.xlsx
@@ -520,7 +520,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Codici dei pericoli a due cifre (es. 1.01) per non confondersi con quelli della prima estrazione.</t>
+          <t>Pericoli secondo il registro interno EN ISO 12100 (prospetto B.1, tre livelli, es. 1.2.1 schiacciamento).</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>7.02 Sostanze – contatto con prodotti (paste abrasive, oli, residui)</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>8.03 Ergonomia – illuminazione o visibilità inadeguata</t>
+          <t>8.2.1 Progettazione errata o insufficiente dell'illuminazione locale sulla macchina</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -1188,8 +1188,8 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>1.10 Meccanico – caduta di oggetti o perdita di stabilità
-1.01 Meccanico – schiacciamento</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)
+1.2.1 Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -1304,8 +1304,9 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>8.04 Ergonomia – errore umano su comandi e segnali
-8.01 Ergonomia – postura scorretta o movimenti ripetitivi</t>
+          <t>8.1.1 Posture incongrue, faticose o sforzi fisici eccessivi
+8.1.2 Movimenti ripetitivi o inadeguata considerazione dell'anatomia della mano/braccio
+8.2.2 Sovraccarico mentale, stress o affaticamento da cattiva progettazione dell'interfaccia (HMI)</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
@@ -1494,7 +1495,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>1.10 Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -1608,7 +1609,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>1.03 Meccanico – taglio</t>
+          <t>1.2.3 Pericolo di taglio o di sezionamento</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1717,8 +1718,8 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>10.01 Combinazione – interazione tra le parti di un insieme
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+10.1.1 Rischi generati dall'azione simultanea di più fattori (es. vibrazioni + freddo + postura)</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1833,8 +1834,8 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-2.02 Elettrico – contatto indiretto (parti in tensione per guasto)</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+2.1.2 Contatto elettrico indiretto (con parti andate in tensione per un guasto)</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1948,8 +1949,8 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>4.01 Rumore – esposizione con danno all'udito
-4.02 Rumore – mancata percezione di segnali e comunicazioni</t>
+          <t>4.1.1 Perdita dell'udito (ipoacusia da trauma acustico o esposizione prolungata)
+4.2.2 Interferenza con la comunicazione verbale e mascheramento dei segnali acustici</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -2064,7 +2065,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>9.01 Ambiente – scivolamento o inciampo</t>
+          <t>9.2.2 Rischio di scivolamento, inciampo o caduta a causa della conformazione dei piani</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -2179,7 +2180,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -2294,7 +2295,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>9.02 Ambiente – caduta dall'alto</t>
+          <t>9.2.2 Rischio di scivolamento, inciampo o caduta a causa della conformazione dei piani</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
@@ -2487,8 +2488,8 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>10.03 Combinazione – manomissione o corruzione del software
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+10.1.1 Rischi generati dall'azione simultanea di più fattori (es. vibrazioni + freddo + postura)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -2604,8 +2605,8 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>10.02 Combinazione – guasto o avaria del sistema di comando
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+10.1.1 Rischi generati dall'azione simultanea di più fattori (es. vibrazioni + freddo + postura)</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -2720,7 +2721,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>8.04 Ergonomia – errore umano su comandi e segnali</t>
+          <t>8.2.2 Sovraccarico mentale, stress o affaticamento da cattiva progettazione dell'interfaccia (HMI)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
@@ -2835,7 +2836,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -2949,7 +2950,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
@@ -3062,7 +3063,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
@@ -3176,8 +3177,8 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.01 Meccanico – schiacciamento</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.1 Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
@@ -3291,7 +3292,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>10.01 Combinazione – interazione tra le parti di un insieme</t>
+          <t>10.1.1 Rischi generati dall'azione simultanea di più fattori (es. vibrazioni + freddo + postura)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -3405,8 +3406,8 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.06 Meccanico – urto</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -3521,8 +3522,8 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.10 Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)
+1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
@@ -3636,8 +3637,8 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.06 Meccanico – urto</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -3825,8 +3826,8 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.06 Meccanico – urto</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
@@ -3939,9 +3940,9 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.06 Meccanico – urto
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -4056,8 +4057,8 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.06 Meccanico – urto</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
@@ -4171,7 +4172,8 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>1.09 Meccanico – proiezione di oggetti o frammenti</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.1.6 Resistenza meccanica insufficiente degli elementi (rotture, cedimenti)</t>
         </is>
       </c>
       <c r="K33" s="2" t="n">
@@ -4284,8 +4286,8 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>9.03 Ambiente – persona chiusa all'interno della macchina
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K34" s="2" t="n">
@@ -4400,8 +4402,8 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.02 Meccanico – cesoiamento</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.2 Pericolo di cesoiamento</t>
         </is>
       </c>
       <c r="K35" s="2" t="n">
@@ -4516,8 +4518,8 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.06 Meccanico – urto</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K36" s="2" t="n">
@@ -4631,8 +4633,8 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>8.01 Ergonomia – postura scorretta o movimenti ripetitivi
-8.02 Ergonomia – movimentazione manuale di carichi</t>
+          <t>8.1.1 Posture incongrue, faticose o sforzi fisici eccessivi
+8.1.2 Movimenti ripetitivi o inadeguata considerazione dell'anatomia della mano/braccio</t>
         </is>
       </c>
       <c r="K37" s="2" t="n">
@@ -4746,8 +4748,8 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>1.10 Meccanico – caduta di oggetti o perdita di stabilità
-1.01 Meccanico – schiacciamento</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)
+1.2.1 Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="K38" s="2" t="n">
@@ -4857,7 +4859,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>3.01 Termico – contatto con superfici o pezzi caldi</t>
+          <t>3.1.1 Ustioni e scottature da contatto con oggetti o fluidi caldi, fiamme o esplosioni</t>
         </is>
       </c>
       <c r="K39" s="2" t="n">
@@ -4971,7 +4973,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>7.01 Sostanze – inalazione di polveri (metalli, abrasivi, fibre)</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K40" s="2" t="n">
@@ -5087,7 +5089,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>3.02 Termico – incendio</t>
+          <t>7.2.1 Pericoli di incendio o combustione di materiali lavorati o fluidi di processo</t>
         </is>
       </c>
       <c r="K41" s="2" t="n">
@@ -5202,7 +5204,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>7.03 Sostanze – esplosione di polveri</t>
+          <t>7.2.2 Pericoli di esplosione (miscele di gas o accumuli di polveri combustibili)</t>
         </is>
       </c>
       <c r="K42" s="2" t="n">
@@ -5316,8 +5318,8 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>7.01 Sostanze – inalazione di polveri (metalli, abrasivi, fibre)
-1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
@@ -5432,8 +5434,8 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2.03 Elettrico – fenomeni elettrostatici
-3.02 Termico – incendio</t>
+          <t>2.2.1 Fenomeni elettrostatici (scosse da cariche statiche accumulate)
+7.2.1 Pericoli di incendio o combustione di materiali lavorati o fluidi di processo</t>
         </is>
       </c>
       <c r="K44" s="2" t="n">
@@ -5542,8 +5544,8 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento
-1.02 Meccanico – cesoiamento</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.2 Pericolo di cesoiamento</t>
         </is>
       </c>
       <c r="K45" s="2" t="n">
@@ -5658,7 +5660,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>1.01 Meccanico – schiacciamento</t>
+          <t>1.2.1 Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="K46" s="2" t="n">
@@ -5771,8 +5773,8 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>8.01 Ergonomia – postura scorretta o movimenti ripetitivi
-8.02 Ergonomia – movimentazione manuale di carichi</t>
+          <t>8.1.1 Posture incongrue, faticose o sforzi fisici eccessivi
+8.1.2 Movimenti ripetitivi o inadeguata considerazione dell'anatomia della mano/braccio</t>
         </is>
       </c>
       <c r="K47" s="2" t="n">
@@ -5881,7 +5883,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>1.10 Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)</t>
         </is>
       </c>
       <c r="K48" s="2" t="n">
@@ -5991,8 +5993,8 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>1.06 Meccanico – urto
-1.01 Meccanico – schiacciamento</t>
+          <t>1.2.1 Pericolo di schiacciamento
+1.2.6 Pericolo di urto</t>
         </is>
       </c>
       <c r="K49" s="2" t="n">
@@ -6106,8 +6108,8 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>1.04 Meccanico – trascinamento o intrappolamento
-1.05 Meccanico – impigliamento</t>
+          <t>1.2.4 Pericolo di impigliamento
+1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K50" s="2" t="n">
@@ -6220,8 +6222,8 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>1.07 Meccanico – abrasione o attrito
-1.04 Meccanico – trascinamento o intrappolamento</t>
+          <t>1.2.5 Pericolo di trascinamento o d'intrappolamento
+1.2.8 Pericolo di attrito o di abrasione</t>
         </is>
       </c>
       <c r="K51" s="2" t="n">
@@ -6336,7 +6338,8 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>1.09 Meccanico – proiezione di oggetti o frammenti</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.1.6 Resistenza meccanica insufficiente degli elementi (rotture, cedimenti)</t>
         </is>
       </c>
       <c r="K52" s="2" t="n">
@@ -6451,8 +6454,8 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.10 Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)
+1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K53" s="2" t="n">
@@ -6566,7 +6569,8 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>1.09 Meccanico – proiezione di oggetti o frammenti</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.1.6 Resistenza meccanica insufficiente degli elementi (rotture, cedimenti)</t>
         </is>
       </c>
       <c r="K54" s="2" t="n">
@@ -6680,7 +6684,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>3.01 Termico – contatto con superfici o pezzi caldi</t>
+          <t>3.1.1 Ustioni e scottature da contatto con oggetti o fluidi caldi, fiamme o esplosioni</t>
         </is>
       </c>
       <c r="K55" s="2" t="n">
@@ -6793,7 +6797,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K56" s="2" t="n">
@@ -6907,8 +6911,8 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>1.04 Meccanico – trascinamento o intrappolamento
-1.05 Meccanico – impigliamento</t>
+          <t>1.2.4 Pericolo di impigliamento
+1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K57" s="2" t="n">
@@ -7021,7 +7025,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>1.04 Meccanico – trascinamento o intrappolamento</t>
+          <t>1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K58" s="2" t="n">
@@ -7135,7 +7139,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>1.04 Meccanico – trascinamento o intrappolamento</t>
+          <t>1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K59" s="2" t="n">
@@ -7248,7 +7252,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>3.01 Termico – contatto con superfici o pezzi caldi</t>
+          <t>3.1.1 Ustioni e scottature da contatto con oggetti o fluidi caldi, fiamme o esplosioni</t>
         </is>
       </c>
       <c r="K60" s="2" t="n">
@@ -7362,8 +7366,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>7.01 Sostanze – inalazione di polveri (metalli, abrasivi, fibre)
-7.04 Sostanze – inalazione di nebbie o vapori</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K61" s="2" t="n">
@@ -7478,7 +7481,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>3.02 Termico – incendio</t>
+          <t>7.2.1 Pericoli di incendio o combustione di materiali lavorati o fluidi di processo</t>
         </is>
       </c>
       <c r="K62" s="2" t="n">
@@ -7593,7 +7596,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>7.03 Sostanze – esplosione di polveri</t>
+          <t>7.2.2 Pericoli di esplosione (miscele di gas o accumuli di polveri combustibili)</t>
         </is>
       </c>
       <c r="K63" s="2" t="n">
@@ -7707,8 +7710,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>7.01 Sostanze – inalazione di polveri (metalli, abrasivi, fibre)
-7.02 Sostanze – contatto con prodotti (paste abrasive, oli, residui)</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K64" s="2" t="n">
@@ -7822,9 +7824,9 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>1.05 Meccanico – impigliamento
-1.04 Meccanico – trascinamento o intrappolamento
-1.07 Meccanico – abrasione o attrito</t>
+          <t>1.2.4 Pericolo di impigliamento
+1.2.5 Pericolo di trascinamento o d'intrappolamento
+1.2.8 Pericolo di attrito o di abrasione</t>
         </is>
       </c>
       <c r="K65" s="2" t="n">
@@ -7938,8 +7940,8 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>1.04 Meccanico – trascinamento o intrappolamento
-1.05 Meccanico – impigliamento</t>
+          <t>1.2.4 Pericolo di impigliamento
+1.2.5 Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="K66" s="2" t="n">
@@ -8052,7 +8054,8 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>1.09 Meccanico – proiezione di oggetti o frammenti</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.1.6 Resistenza meccanica insufficiente degli elementi (rotture, cedimenti)</t>
         </is>
       </c>
       <c r="K67" s="2" t="n">
@@ -8167,8 +8170,8 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.01 Meccanico – schiacciamento</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.1 Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="K68" s="2" t="n">
@@ -8282,8 +8285,8 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.05 Meccanico – impigliamento</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.4 Pericolo di impigliamento</t>
         </is>
       </c>
       <c r="K69" s="2" t="n">
@@ -8397,7 +8400,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>3.01 Termico – contatto con superfici o pezzi caldi</t>
+          <t>3.1.1 Ustioni e scottature da contatto con oggetti o fluidi caldi, fiamme o esplosioni</t>
         </is>
       </c>
       <c r="K70" s="2" t="n">
@@ -8510,7 +8513,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2.01 Elettrico – contatto diretto con parti attive</t>
+          <t>2.1.1 Contatto elettrico diretto (con parti normalmente in tensione)</t>
         </is>
       </c>
       <c r="K71" s="2" t="n">
@@ -8625,7 +8628,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2.02 Elettrico – contatto indiretto (parti in tensione per guasto)</t>
+          <t>2.1.2 Contatto elettrico indiretto (con parti andate in tensione per un guasto)</t>
         </is>
       </c>
       <c r="K72" s="2" t="n">
@@ -8740,8 +8743,8 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-2.01 Elettrico – contatto diretto con parti attive</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+2.1.1 Contatto elettrico diretto (con parti normalmente in tensione)</t>
         </is>
       </c>
       <c r="K73" s="2" t="n">
@@ -8855,8 +8858,8 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2.04 Elettrico – cortocircuito o sovraccarico con innesco di incendio
-3.02 Termico – incendio</t>
+          <t>2.2.2 Irraggiamento termico o proiezioni da cortocircuiti
+7.2.1 Pericoli di incendio o combustione di materiali lavorati o fluidi di processo</t>
         </is>
       </c>
       <c r="K74" s="2" t="n">
@@ -8965,7 +8968,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>1.11 Meccanico – fluidi in pressione</t>
+          <t>1.2.9 Pericolo di eiezione o iniezione di fluido ad alta pressione</t>
         </is>
       </c>
       <c r="K75" s="2" t="n">
@@ -9075,8 +9078,8 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.11 Meccanico – fluidi in pressione</t>
+          <t>1.1.4 Massa e velocità (energia cinetica di elementi in movimento)
+1.2.9 Pericolo di eiezione o iniezione di fluido ad alta pressione</t>
         </is>
       </c>
       <c r="K76" s="2" t="n">
@@ -9190,8 +9193,8 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>1.12 Meccanico – movimento o avviamento inatteso
-1.10 Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>1.1.3 Massa e stabilità (energia potenziale dovuta alla gravità)
+1.1.4 Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="K77" s="2" t="n">
@@ -9300,7 +9303,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>4.01 Rumore – esposizione con danno all'udito</t>
+          <t>4.1.1 Perdita dell'udito (ipoacusia da trauma acustico o esposizione prolungata)</t>
         </is>
       </c>
       <c r="K78" s="2" t="n">
@@ -9409,8 +9412,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>7.02 Sostanze – contatto con prodotti (paste abrasive, oli, residui)
-7.04 Sostanze – inalazione di nebbie o vapori</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K79" s="2" t="n">
@@ -9524,8 +9526,8 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>1.11 Meccanico – fluidi in pressione
-7.02 Sostanze – contatto con prodotti (paste abrasive, oli, residui)</t>
+          <t>1.2.9 Pericolo di eiezione o iniezione di fluido ad alta pressione
+7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K80" s="2" t="n">
@@ -9639,7 +9641,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>7.02 Sostanze – contatto con prodotti (paste abrasive, oli, residui)</t>
+          <t>7.1.1 Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="K81" s="2" t="n">
@@ -9753,7 +9755,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>9.01 Ambiente – scivolamento o inciampo</t>
+          <t>9.2.2 Rischio di scivolamento, inciampo o caduta a causa della conformazione dei piani</t>
         </is>
       </c>
       <c r="K82" s="2" t="n">
@@ -9862,7 +9864,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>8.04 Ergonomia – errore umano su comandi e segnali</t>
+          <t>8.2.2 Sovraccarico mentale, stress o affaticamento da cattiva progettazione dell'interfaccia (HMI)</t>
         </is>
       </c>
       <c r="K83" s="2" t="n">
@@ -9971,8 +9973,8 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>4.02 Rumore – mancata percezione di segnali e comunicazioni
-8.04 Ergonomia – errore umano su comandi e segnali</t>
+          <t>4.2.2 Interferenza con la comunicazione verbale e mascheramento dei segnali acustici
+8.2.2 Sovraccarico mentale, stress o affaticamento da cattiva progettazione dell'interfaccia (HMI)</t>
         </is>
       </c>
       <c r="K84" s="2" t="n">
@@ -19310,7 +19312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19338,207 +19340,207 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Meccanico – schiacciamento</t>
+          <t>Forma (elementi taglienti, spigoli vivi, pezzi aguzzi)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>1.1.2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Meccanico – cesoiamento</t>
+          <t>Posizione relativa (zone di convergenza o ridotti spazi tra parti mobili)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.1.3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Meccanico – taglio</t>
+          <t>Massa e stabilità (energia potenziale dovuta alla gravità)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.1.4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Meccanico – trascinamento o intrappolamento</t>
+          <t>Massa e velocità (energia cinetica di elementi in movimento)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>1.1.5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Meccanico – impigliamento</t>
+          <t>Accelerazione o decelerazione inadeguata</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.1.6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Meccanico – urto</t>
+          <t>Resistenza meccanica insufficiente degli elementi (rotture, cedimenti)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Meccanico – abrasione o attrito</t>
+          <t>Pericolo di schiacciamento</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Meccanico – perforazione o puntura</t>
+          <t>Pericolo di cesoiamento</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Meccanico – proiezione di oggetti o frammenti</t>
+          <t>Pericolo di taglio o di sezionamento</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Meccanico – caduta di oggetti o perdita di stabilità</t>
+          <t>Pericolo di impigliamento</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.2.5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Meccanico – fluidi in pressione</t>
+          <t>Pericolo di trascinamento o d'intrappolamento</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Meccanico – movimento o avviamento inatteso</t>
+          <t>Pericolo di urto</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.2.7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Elettrico – contatto diretto con parti attive</t>
+          <t>Pericolo di perforazione o di puntura</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.2.8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Elettrico – contatto indiretto (parti in tensione per guasto)</t>
+          <t>Pericolo di attrito o di abrasione</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -19548,102 +19550,102 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.2.9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Elettrico – fenomeni elettrostatici</t>
+          <t>Pericolo di eiezione o iniezione di fluido ad alta pressione</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>2.1.1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Elettrico – cortocircuito o sovraccarico con innesco di incendio</t>
+          <t>Contatto elettrico diretto (con parti normalmente in tensione)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>2.1.2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Termico – contatto con superfici o pezzi caldi</t>
+          <t>Contatto elettrico indiretto (con parti andate in tensione per un guasto)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>2.1.3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Termico – incendio</t>
+          <t>Avvicinamento a parti sotto alta tensione (effetto arco elettrico)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4.01</t>
+          <t>2.2.1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Rumore – esposizione con danno all'udito</t>
+          <t>Fenomeni elettrostatici (scosse da cariche statiche accumulate)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>2.2.2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Rumore – mancata percezione di segnali e comunicazioni</t>
+          <t>Irraggiamento termico o proiezioni da cortocircuiti</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7.01</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sostanze – inalazione di polveri (metalli, abrasivi, fibre)</t>
+          <t>Ustioni e scottature da contatto con oggetti o fluidi caldi, fiamme o esplosioni</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -19653,42 +19655,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7.02</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sostanze – contatto con prodotti (paste abrasive, oli, residui)</t>
+          <t>Lesioni da contatto con superfici o fluidi a temperatura estremamente bassa (congelamento)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7.03</t>
+          <t>3.2.1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sostanze – esplosione di polveri</t>
+          <t>Danni alla salute causati da un ambiente di lavoro eccessivamente caldo o freddo</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7.04</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sostanze – inalazione di nebbie o vapori</t>
+          <t>Perdita dell'udito (ipoacusia da trauma acustico o esposizione prolungata)</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -19698,151 +19700,331 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8.01</t>
+          <t>4.1.2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ergonomia – postura scorretta o movimenti ripetitivi</t>
+          <t>Acufene (ronzio o fischio permanente nelle orecchie)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8.02</t>
+          <t>4.2.1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ergonomia – movimentazione manuale di carichi</t>
+          <t>Disturbi dell'equilibrio o senso di vertigine</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8.03</t>
+          <t>4.2.2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ergonomia – illuminazione o visibilità inadeguata</t>
+          <t>Interferenza con la comunicazione verbale e mascheramento dei segnali acustici</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8.04</t>
+          <t>5.1.1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ergonomia – errore umano su comandi e segnali</t>
+          <t>Sindrome da vibrazioni mano-braccio (disturbi vascolari, neurologici e ossei)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9.01</t>
+          <t>5.1.2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ambiente – scivolamento o inciampo</t>
+          <t>Sindrome da vibrazioni corpo intero (traumi alla colonna vertebrale, lombalgie)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9.02</t>
+          <t>6.1.1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ambiente – caduta dall'alto</t>
+          <t>Radiazioni ionizzanti (fonti di raggi X, raggi gamma o particelle)</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9.03</t>
+          <t>6.1.2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ambiente – persona chiusa all'interno della macchina</t>
+          <t>Campi elettromagnetici (unità CEM a bassa o alta frequenza)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10.01</t>
+          <t>6.2.1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Combinazione – interazione tra le parti di un insieme</t>
+          <t>Radiazioni ottiche artificiali (ROA): infrarossi, luce visibile estrema, ultravioletti</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>10.02</t>
+          <t>6.2.2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Combinazione – guasto o avaria del sistema di comando</t>
+          <t>Radiazioni laser (danni irreversibili a occhi e pelle)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>10.03</t>
+          <t>7.1.1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Combinazione – manomissione o corruzione del software</t>
+          <t>Pericoli tossici o nocivi per inalazione, ingestione o contatto con elementi chimici</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>7.1.2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pericoli biologici o microbiologici (esposizione a virus o batteri nei liquidi)</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>7.2.1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pericoli di incendio o combustione di materiali lavorati o fluidi di processo</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>7.2.2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Pericoli di esplosione (miscele di gas o accumuli di polveri combustibili)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>8.1.1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Posture incongrue, faticose o sforzi fisici eccessivi</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>8.1.2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Movimenti ripetitivi o inadeguata considerazione dell'anatomia della mano/braccio</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>8.2.1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Progettazione errata o insufficiente dell'illuminazione locale sulla macchina</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>8.2.2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sovraccarico mentale, stress o affaticamento da cattiva progettazione dell'interfaccia (HMI)</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>9.1.1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Fulminazione da scariche atmosferiche esterne</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>9.1.2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Condizioni meteorologiche estreme (vento forte, neve, temperature proibitive)</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>9.2.1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Mancanza di stabilità del suolo o pendenze (rischio di ribaltamento)</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>9.2.2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Rischio di scivolamento, inciampo o caduta a causa della conformazione dei piani</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>10.1.1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Rischi generati dall'azione simultanea di più fattori (es. vibrazioni + freddo + postura)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>